<commit_message>
Added OpenPo & Amend Test Scenarios, PO Amend Test SCeanrios
Added OpenPo & Amend Test Scenarios, PO Amend Test SCeanrios
</commit_message>
<xml_diff>
--- a/testdata/OpenPOSheet.xlsx
+++ b/testdata/OpenPOSheet.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="66">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>18</t>
+  </si>
+  <si>
+    <t>TVS-SIM-349399</t>
   </si>
 </sst>
 </file>
@@ -1352,39 +1355,39 @@
   <dimension ref="A1:AO16"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.8518518518519" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.5740740740741" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.8518518518519" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.287037037037" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="12" max="12" width="17.8518518518519" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="14" max="14" width="18" style="2" customWidth="1"/>
-    <col min="15" max="15" width="18.1388888888889" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.287037037037" style="2" customWidth="1"/>
-    <col min="17" max="17" width="19" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.287037037037" style="2" customWidth="1"/>
-    <col min="19" max="19" width="10.712962962963" style="2" customWidth="1"/>
-    <col min="20" max="20" width="12.1388888888889" style="2" customWidth="1"/>
-    <col min="21" max="21" width="20.5740740740741" style="2" customWidth="1"/>
-    <col min="22" max="22" width="28.712962962963" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.28703703703704" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10" style="2" customWidth="1"/>
-    <col min="25" max="26" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="27" max="27" width="11.712962962963" style="2" customWidth="1"/>
-    <col min="28" max="32" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="33" max="35" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="36" max="36" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="37" max="39" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="40" max="40" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="41" max="41" width="23.287037037037" style="2" customWidth="1"/>
-    <col min="42" max="16384" width="9.13888888888889" style="2"/>
+    <col min="1" max="1" customWidth="true" style="2" width="8.0"/>
+    <col min="2" max="2" customWidth="true" style="2" width="21.0"/>
+    <col min="3" max="3" customWidth="true" style="2" width="21.8518518518519"/>
+    <col min="4" max="4" customWidth="true" style="2" width="10.0"/>
+    <col min="5" max="5" customWidth="true" style="2" width="12.5740740740741"/>
+    <col min="6" max="6" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="7" max="7" customWidth="true" style="2" width="10.1388888888889"/>
+    <col min="8" max="8" customWidth="true" style="2" width="11.8518518518519"/>
+    <col min="9" max="9" customWidth="true" style="2" width="14.4259259259259"/>
+    <col min="10" max="10" customWidth="true" style="2" width="18.287037037037"/>
+    <col min="11" max="11" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="12" max="12" customWidth="true" style="2" width="17.8518518518519"/>
+    <col min="13" max="13" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="14" max="14" customWidth="true" style="2" width="18.0"/>
+    <col min="15" max="15" customWidth="true" style="2" width="18.1388888888889"/>
+    <col min="16" max="16" customWidth="true" style="2" width="20.287037037037"/>
+    <col min="17" max="17" customWidth="true" style="2" width="19.0"/>
+    <col min="18" max="18" customWidth="true" style="2" width="13.287037037037"/>
+    <col min="19" max="19" customWidth="true" style="2" width="10.712962962963"/>
+    <col min="20" max="20" customWidth="true" style="2" width="12.1388888888889"/>
+    <col min="21" max="21" customWidth="true" style="2" width="20.5740740740741"/>
+    <col min="22" max="22" customWidth="true" style="2" width="28.712962962963"/>
+    <col min="23" max="23" customWidth="true" style="2" width="9.28703703703704"/>
+    <col min="24" max="24" customWidth="true" style="2" width="10.0"/>
+    <col min="25" max="26" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="27" max="27" customWidth="true" style="2" width="11.712962962963"/>
+    <col min="28" max="32" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="33" max="35" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="36" max="36" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="37" max="39" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="40" max="40" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="41" max="41" customWidth="true" style="2" width="23.287037037037"/>
+    <col min="42" max="16384" style="2" width="9.13888888888889"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:41">
@@ -2969,39 +2972,39 @@
   <dimension ref="A1:AO16"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" customWidth="1"/>
-    <col min="2" max="2" width="27.5740740740741" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.1388888888889" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.5740740740741" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.8518518518519" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.287037037037" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="12" max="12" width="17.8518518518519" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="14" max="14" width="18" style="2" customWidth="1"/>
-    <col min="15" max="15" width="18.1388888888889" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.287037037037" style="2" customWidth="1"/>
-    <col min="17" max="17" width="19" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.287037037037" style="2" customWidth="1"/>
-    <col min="19" max="19" width="10.712962962963" style="2" customWidth="1"/>
-    <col min="20" max="20" width="12.1388888888889" style="2" customWidth="1"/>
-    <col min="21" max="21" width="20.5740740740741" style="2" customWidth="1"/>
-    <col min="22" max="22" width="28.712962962963" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.28703703703704" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10" style="2" customWidth="1"/>
-    <col min="25" max="26" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="27" max="27" width="11.712962962963" style="2" customWidth="1"/>
-    <col min="28" max="32" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="33" max="35" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="36" max="36" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="37" max="39" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="40" max="40" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="41" max="41" width="23.287037037037" style="2" customWidth="1"/>
-    <col min="42" max="16384" width="9.13888888888889" style="2"/>
+    <col min="1" max="1" customWidth="true" style="2" width="8.0"/>
+    <col min="2" max="2" customWidth="true" style="2" width="27.5740740740741"/>
+    <col min="3" max="3" customWidth="true" style="2" width="33.1388888888889"/>
+    <col min="4" max="4" customWidth="true" style="2" width="10.0"/>
+    <col min="5" max="5" customWidth="true" style="2" width="12.5740740740741"/>
+    <col min="6" max="6" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="7" max="7" customWidth="true" style="2" width="10.1388888888889"/>
+    <col min="8" max="8" customWidth="true" style="2" width="11.8518518518519"/>
+    <col min="9" max="9" customWidth="true" style="2" width="14.4259259259259"/>
+    <col min="10" max="10" customWidth="true" style="2" width="18.287037037037"/>
+    <col min="11" max="11" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="12" max="12" customWidth="true" style="2" width="17.8518518518519"/>
+    <col min="13" max="13" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="14" max="14" customWidth="true" style="2" width="18.0"/>
+    <col min="15" max="15" customWidth="true" style="2" width="18.1388888888889"/>
+    <col min="16" max="16" customWidth="true" style="2" width="20.287037037037"/>
+    <col min="17" max="17" customWidth="true" style="2" width="19.0"/>
+    <col min="18" max="18" customWidth="true" style="2" width="13.287037037037"/>
+    <col min="19" max="19" customWidth="true" style="2" width="10.712962962963"/>
+    <col min="20" max="20" customWidth="true" style="2" width="12.1388888888889"/>
+    <col min="21" max="21" customWidth="true" style="2" width="20.5740740740741"/>
+    <col min="22" max="22" customWidth="true" style="2" width="28.712962962963"/>
+    <col min="23" max="23" customWidth="true" style="2" width="9.28703703703704"/>
+    <col min="24" max="24" customWidth="true" style="2" width="10.0"/>
+    <col min="25" max="26" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="27" max="27" customWidth="true" style="2" width="11.712962962963"/>
+    <col min="28" max="32" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="33" max="35" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="36" max="36" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="37" max="39" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="40" max="40" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="41" max="41" customWidth="true" style="2" width="23.287037037037"/>
+    <col min="42" max="16384" style="2" width="9.13888888888889"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:41">
@@ -4586,39 +4589,39 @@
   <dimension ref="A1:AO16"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" customWidth="1"/>
-    <col min="2" max="2" width="27.5740740740741" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.1388888888889" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.5740740740741" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.8518518518519" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.287037037037" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="12" max="12" width="17.8518518518519" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="14" max="14" width="18" style="2" customWidth="1"/>
-    <col min="15" max="15" width="18.1388888888889" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.287037037037" style="2" customWidth="1"/>
-    <col min="17" max="17" width="19" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.287037037037" style="2" customWidth="1"/>
-    <col min="19" max="19" width="10.712962962963" style="2" customWidth="1"/>
-    <col min="20" max="20" width="12.1388888888889" style="2" customWidth="1"/>
-    <col min="21" max="21" width="20.5740740740741" style="2" customWidth="1"/>
-    <col min="22" max="22" width="28.712962962963" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.28703703703704" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10" style="2" customWidth="1"/>
-    <col min="25" max="26" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="27" max="27" width="11.712962962963" style="2" customWidth="1"/>
-    <col min="28" max="32" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="33" max="35" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="36" max="36" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="37" max="39" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="40" max="40" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="41" max="41" width="23.287037037037" style="2" customWidth="1"/>
-    <col min="42" max="16384" width="9.13888888888889" style="2"/>
+    <col min="1" max="1" customWidth="true" style="2" width="8.0"/>
+    <col min="2" max="2" customWidth="true" style="2" width="27.5740740740741"/>
+    <col min="3" max="3" customWidth="true" style="2" width="33.1388888888889"/>
+    <col min="4" max="4" customWidth="true" style="2" width="10.0"/>
+    <col min="5" max="5" customWidth="true" style="2" width="12.5740740740741"/>
+    <col min="6" max="6" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="7" max="7" customWidth="true" style="2" width="10.1388888888889"/>
+    <col min="8" max="8" customWidth="true" style="2" width="11.8518518518519"/>
+    <col min="9" max="9" customWidth="true" style="2" width="14.4259259259259"/>
+    <col min="10" max="10" customWidth="true" style="2" width="18.287037037037"/>
+    <col min="11" max="11" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="12" max="12" customWidth="true" style="2" width="17.8518518518519"/>
+    <col min="13" max="13" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="14" max="14" customWidth="true" style="2" width="18.0"/>
+    <col min="15" max="15" customWidth="true" style="2" width="18.1388888888889"/>
+    <col min="16" max="16" customWidth="true" style="2" width="20.287037037037"/>
+    <col min="17" max="17" customWidth="true" style="2" width="19.0"/>
+    <col min="18" max="18" customWidth="true" style="2" width="13.287037037037"/>
+    <col min="19" max="19" customWidth="true" style="2" width="10.712962962963"/>
+    <col min="20" max="20" customWidth="true" style="2" width="12.1388888888889"/>
+    <col min="21" max="21" customWidth="true" style="2" width="20.5740740740741"/>
+    <col min="22" max="22" customWidth="true" style="2" width="28.712962962963"/>
+    <col min="23" max="23" customWidth="true" style="2" width="9.28703703703704"/>
+    <col min="24" max="24" customWidth="true" style="2" width="10.0"/>
+    <col min="25" max="26" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="27" max="27" customWidth="true" style="2" width="11.712962962963"/>
+    <col min="28" max="32" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="33" max="35" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="36" max="36" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="37" max="39" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="40" max="40" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="41" max="41" customWidth="true" style="2" width="23.287037037037"/>
+    <col min="42" max="16384" style="2" width="9.13888888888889"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:41">
@@ -6203,39 +6206,39 @@
   <dimension ref="A1:AO5"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="13.8" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.8518518518519" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.5740740740741" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.8518518518519" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.287037037037" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="12" max="12" width="17.8518518518519" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.8518518518519" style="2" customWidth="1"/>
-    <col min="14" max="14" width="18" style="2" customWidth="1"/>
-    <col min="15" max="15" width="18.1388888888889" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.287037037037" style="2" customWidth="1"/>
-    <col min="17" max="17" width="19" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.287037037037" style="2" customWidth="1"/>
-    <col min="19" max="19" width="10.712962962963" style="2" customWidth="1"/>
-    <col min="20" max="20" width="12.1388888888889" style="2" customWidth="1"/>
-    <col min="21" max="21" width="20.5740740740741" style="2" customWidth="1"/>
-    <col min="22" max="22" width="28.712962962963" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.28703703703704" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10" style="2" customWidth="1"/>
-    <col min="25" max="26" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="27" max="27" width="11.712962962963" style="2" customWidth="1"/>
-    <col min="28" max="32" width="11.5740740740741" style="2" customWidth="1"/>
-    <col min="33" max="35" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="36" max="36" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="37" max="39" width="12.287037037037" style="2" customWidth="1"/>
-    <col min="40" max="40" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="41" max="41" width="23.287037037037" style="2" customWidth="1"/>
-    <col min="42" max="16384" width="9.13888888888889" style="2"/>
+    <col min="1" max="1" customWidth="true" style="2" width="8.0"/>
+    <col min="2" max="2" customWidth="true" style="2" width="21.0"/>
+    <col min="3" max="3" customWidth="true" style="2" width="21.8518518518519"/>
+    <col min="4" max="4" customWidth="true" style="2" width="10.0"/>
+    <col min="5" max="5" customWidth="true" style="2" width="12.5740740740741"/>
+    <col min="6" max="6" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="7" max="7" customWidth="true" style="2" width="10.1388888888889"/>
+    <col min="8" max="8" customWidth="true" style="2" width="11.8518518518519"/>
+    <col min="9" max="9" customWidth="true" style="2" width="14.4259259259259"/>
+    <col min="10" max="10" customWidth="true" style="2" width="18.287037037037"/>
+    <col min="11" max="11" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="12" max="12" customWidth="true" style="2" width="17.8518518518519"/>
+    <col min="13" max="13" customWidth="true" style="2" width="12.8518518518519"/>
+    <col min="14" max="14" customWidth="true" style="2" width="18.0"/>
+    <col min="15" max="15" customWidth="true" style="2" width="18.1388888888889"/>
+    <col min="16" max="16" customWidth="true" style="2" width="20.287037037037"/>
+    <col min="17" max="17" customWidth="true" style="2" width="19.0"/>
+    <col min="18" max="18" customWidth="true" style="2" width="13.287037037037"/>
+    <col min="19" max="19" customWidth="true" style="2" width="10.712962962963"/>
+    <col min="20" max="20" customWidth="true" style="2" width="12.1388888888889"/>
+    <col min="21" max="21" customWidth="true" style="2" width="20.5740740740741"/>
+    <col min="22" max="22" customWidth="true" style="2" width="28.712962962963"/>
+    <col min="23" max="23" customWidth="true" style="2" width="9.28703703703704"/>
+    <col min="24" max="24" customWidth="true" style="2" width="10.0"/>
+    <col min="25" max="26" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="27" max="27" customWidth="true" style="2" width="11.712962962963"/>
+    <col min="28" max="32" customWidth="true" style="2" width="11.5740740740741"/>
+    <col min="33" max="35" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="36" max="36" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="37" max="39" customWidth="true" style="2" width="12.287037037037"/>
+    <col min="40" max="40" customWidth="true" style="2" width="14.712962962963"/>
+    <col min="41" max="41" customWidth="true" style="2" width="23.287037037037"/>
+    <col min="42" max="16384" style="2" width="9.13888888888889"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:41">
@@ -6475,11 +6478,11 @@
       <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>60</v>
+      <c r="B4" t="s" s="2">
+        <v>65</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>65</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>51</v>
@@ -6487,17 +6490,17 @@
       <c r="E4" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" t="s" s="2">
         <v>62</v>
       </c>
       <c r="H4" s="12">
         <f>F4*G4</f>
         <v>750</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" t="s" s="2">
         <v>61</v>
       </c>
       <c r="J4" s="12"/>
@@ -6534,10 +6537,10 @@
         <f>(H4-R4)</f>
         <v>712.5</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="T4" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="U4" t="s" s="2">
         <v>64</v>
       </c>
       <c r="V4" s="19">

</xml_diff>